<commit_message>
created class with contact with phone
</commit_message>
<xml_diff>
--- a/ComcastCRMGUIFramework/testdata/Book1.xlsx
+++ b/ComcastCRMGUIFramework/testdata/Book1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\eclipse-workspace\ComcastCRMGUIFramework\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\git\repository\ComcastCRMGUIFramework\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8DC0042-2244-4D8F-8E64-ED5E691A7BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A07F4678-C17C-4BE3-9CC0-869DD312DEC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{10676D73-7227-40E6-B18E-A2FC50E405D8}"/>
+    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{10676D73-7227-40E6-B18E-A2FC50E405D8}"/>
   </bookViews>
   <sheets>
     <sheet name="org" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="30">
   <si>
     <t>Test_ID</t>
   </si>
@@ -108,6 +108,15 @@
   </si>
   <si>
     <t>Apple iPhone 15 Plus (128 GB) - Blue</t>
+  </si>
+  <si>
+    <t>create contact with phone</t>
+  </si>
+  <si>
+    <t>8070605040</t>
+  </si>
+  <si>
+    <t>9000020000</t>
   </si>
 </sst>
 </file>
@@ -603,8 +612,8 @@
       <c r="C2" t="s">
         <v>20</v>
       </c>
-      <c r="D2">
-        <v>9000010010</v>
+      <c r="D2" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -632,13 +641,13 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
         <v>11</v>
       </c>
-      <c r="D5">
-        <v>8070605040</v>
+      <c r="D5" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>

</xml_diff>